<commit_message>
add tracker to app
</commit_message>
<xml_diff>
--- a/CTH CALENDER.xlsx
+++ b/CTH CALENDER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Surau-Imam-Attendence-tracker-App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EAADE36D-074F-4D8E-97B9-775BCECAB772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81F4F031-DFE5-48A8-BC54-7D88912452DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="15225" windowHeight="21105" xr2:uid="{D170A22A-6A5D-4A5E-BBEE-B156D0137A28}"/>
+    <workbookView xWindow="-16305" yWindow="14100" windowWidth="16410" windowHeight="14205" xr2:uid="{D170A22A-6A5D-4A5E-BBEE-B156D0137A28}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="6">
   <si>
     <t>IMAM MASRI</t>
   </si>
@@ -51,6 +51,12 @@
   </si>
   <si>
     <t>IMAM ZAHAR</t>
+  </si>
+  <si>
+    <t>IMAM HAZIQ</t>
+  </si>
+  <si>
+    <t>IMAM ARIFIN</t>
   </si>
 </sst>
 </file>
@@ -503,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E62FA82-BEDC-4B79-A05F-533854169D57}">
-  <dimension ref="C2:D20"/>
+  <dimension ref="C2:D27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="3" customWidth="1"/>
@@ -577,10 +583,40 @@
       <c r="D18" s="4"/>
     </row>
     <row r="19" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="D19" s="4"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="5" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="20" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="D20" s="4"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C21" s="3"/>
+      <c r="D21" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C25" s="1"/>
+      <c r="D25" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C26" s="2"/>
+      <c r="D26" s="5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C27" s="3"/>
+      <c r="D27" s="5" t="s">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>